<commit_message>
chore: update hasil pengujian dengan JWT key yang aman (64 byte)
</commit_message>
<xml_diff>
--- a/benchmark/output/hasil_pengujian.xlsx
+++ b/benchmark/output/hasil_pengujian.xlsx
@@ -575,11 +575,11 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>simulasi_gambar.png</t>
+          <t>gambar_uji.png</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>2008</v>
+        <v>116</v>
       </c>
       <c r="D10" t="b">
         <v>1</v>
@@ -591,11 +591,11 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>simulasi_dokumen.pdf</t>
+          <t>dokumen_uji.pdf</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>3009</v>
+        <v>328</v>
       </c>
       <c r="D11" t="b">
         <v>1</v>
@@ -649,10 +649,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>47.785</v>
+        <v>46.769</v>
       </c>
       <c r="D2" t="n">
-        <v>48.707</v>
+        <v>48.598</v>
       </c>
     </row>
     <row r="3">
@@ -667,10 +667,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>34.621</v>
+        <v>37.116</v>
       </c>
       <c r="D3" t="n">
-        <v>49.759</v>
+        <v>54.274</v>
       </c>
     </row>
     <row r="4">
@@ -685,10 +685,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>49.067</v>
+        <v>48.556</v>
       </c>
       <c r="D4" t="n">
-        <v>49.03</v>
+        <v>51.428</v>
       </c>
     </row>
     <row r="5">
@@ -703,10 +703,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>37.384</v>
+        <v>38.114</v>
       </c>
       <c r="D5" t="n">
-        <v>48.611</v>
+        <v>47.4</v>
       </c>
     </row>
     <row r="6">
@@ -721,10 +721,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>60.069</v>
+        <v>61.146</v>
       </c>
       <c r="D6" t="n">
-        <v>63.008</v>
+        <v>65.006</v>
       </c>
     </row>
     <row r="7">
@@ -739,10 +739,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>52.935</v>
+        <v>55.25</v>
       </c>
       <c r="D7" t="n">
-        <v>67.79900000000001</v>
+        <v>69.247</v>
       </c>
     </row>
   </sheetData>
@@ -783,10 +783,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>48.85</v>
+        <v>48.74</v>
       </c>
       <c r="C2" t="n">
-        <v>49.01</v>
+        <v>49.84</v>
       </c>
     </row>
     <row r="3">
@@ -796,10 +796,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>48.74</v>
+        <v>48.95</v>
       </c>
       <c r="C3" t="n">
-        <v>50.84</v>
+        <v>49.79</v>
       </c>
     </row>
   </sheetData>
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>7.9095</v>
+        <v>7.9218</v>
       </c>
     </row>
     <row r="4">
@@ -855,7 +855,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>7.9268</v>
+        <v>7.9065</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
bench: pakai berkas uji asli (gambar_uji.png, dokumen_uji.pdf), perbarui hasil
</commit_message>
<xml_diff>
--- a/benchmark/output/hasil_pengujian.xlsx
+++ b/benchmark/output/hasil_pengujian.xlsx
@@ -579,7 +579,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>209999</v>
+        <v>2718788</v>
       </c>
       <c r="D10" t="b">
         <v>1</v>
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>297944</v>
+        <v>1437108</v>
       </c>
       <c r="D11" t="b">
         <v>1</v>
@@ -649,10 +649,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>54.967</v>
+        <v>88.27</v>
       </c>
       <c r="D2" t="n">
-        <v>49.036</v>
+        <v>94.586</v>
       </c>
     </row>
     <row r="3">
@@ -667,10 +667,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>82.39</v>
+        <v>74.402</v>
       </c>
       <c r="D3" t="n">
-        <v>54.098</v>
+        <v>75.39</v>
       </c>
     </row>
     <row r="4">
@@ -685,10 +685,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>50.52</v>
+        <v>76.354</v>
       </c>
       <c r="D4" t="n">
-        <v>51.194</v>
+        <v>79.583</v>
       </c>
     </row>
     <row r="5">
@@ -703,10 +703,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>38.64</v>
+        <v>61.846</v>
       </c>
       <c r="D5" t="n">
-        <v>55.106</v>
+        <v>69.096</v>
       </c>
     </row>
     <row r="6">
@@ -721,10 +721,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>80.523</v>
+        <v>87.476</v>
       </c>
       <c r="D6" t="n">
-        <v>71.056</v>
+        <v>89.083</v>
       </c>
     </row>
     <row r="7">
@@ -739,10 +739,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>59.466</v>
+        <v>75.661</v>
       </c>
       <c r="D7" t="n">
-        <v>121.61</v>
+        <v>118.531</v>
       </c>
     </row>
   </sheetData>
@@ -867,7 +867,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>7.9162</v>
+        <v>7.926</v>
       </c>
     </row>
     <row r="4">
@@ -877,7 +877,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>7.9189</v>
+        <v>7.9164</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
bench: hitung entropi dan histogram dari berkas uji asli
</commit_message>
<xml_diff>
--- a/benchmark/output/hasil_pengujian.xlsx
+++ b/benchmark/output/hasil_pengujian.xlsx
@@ -649,10 +649,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>88.27</v>
+        <v>92.517</v>
       </c>
       <c r="D2" t="n">
-        <v>94.586</v>
+        <v>92.13</v>
       </c>
     </row>
     <row r="3">
@@ -667,10 +667,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>74.402</v>
+        <v>69.104</v>
       </c>
       <c r="D3" t="n">
-        <v>75.39</v>
+        <v>77.765</v>
       </c>
     </row>
     <row r="4">
@@ -685,10 +685,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>76.354</v>
+        <v>78.492</v>
       </c>
       <c r="D4" t="n">
-        <v>79.583</v>
+        <v>73.931</v>
       </c>
     </row>
     <row r="5">
@@ -703,10 +703,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>61.846</v>
+        <v>62.61</v>
       </c>
       <c r="D5" t="n">
-        <v>69.096</v>
+        <v>73.869</v>
       </c>
     </row>
     <row r="6">
@@ -721,10 +721,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>87.476</v>
+        <v>90.857</v>
       </c>
       <c r="D6" t="n">
-        <v>89.083</v>
+        <v>96.431</v>
       </c>
     </row>
     <row r="7">
@@ -739,10 +739,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>75.661</v>
+        <v>78.32299999999999</v>
       </c>
       <c r="D7" t="n">
-        <v>118.531</v>
+        <v>127.287</v>
       </c>
     </row>
   </sheetData>
@@ -835,7 +835,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -846,6 +846,11 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>Ukuran (byte)</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>Entropi (bit/byte)</t>
         </is>
       </c>
@@ -853,31 +858,157 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Plaintext asli</t>
+          <t>Teks contoh: plainteks</t>
         </is>
       </c>
       <c r="B2" t="n">
+        <v>2140</v>
+      </c>
+      <c r="C2" t="n">
         <v>4.1082</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Cipherteks AES-256-GCM</t>
+          <t>Teks contoh: AES-256-GCM</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>7.926</v>
+        <v>2184</v>
+      </c>
+      <c r="C3" t="n">
+        <v>7.8951</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Cipherteks ChaCha20-Poly1305</t>
+          <t>Teks contoh: ChaCha20-Poly1305</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>7.9164</v>
+        <v>2184</v>
+      </c>
+      <c r="C4" t="n">
+        <v>7.9075</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Piksel mentah gambar_uji: plainteks</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4800000</v>
+      </c>
+      <c r="C5" t="n">
+        <v>7.7106</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Piksel mentah gambar_uji: AES-256-GCM</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>4800044</v>
+      </c>
+      <c r="C6" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Piksel mentah gambar_uji: ChaCha20-Poly1305</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>4800044</v>
+      </c>
+      <c r="C7" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>gambar_uji.png: plainteks</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>2718788</v>
+      </c>
+      <c r="C8" t="n">
+        <v>7.9975</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>gambar_uji.png: AES-256-GCM</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>2718832</v>
+      </c>
+      <c r="C9" t="n">
+        <v>7.9999</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>gambar_uji.png: ChaCha20-Poly1305</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>2718832</v>
+      </c>
+      <c r="C10" t="n">
+        <v>7.9999</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>dokumen_uji.pdf: plainteks</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1437108</v>
+      </c>
+      <c r="C11" t="n">
+        <v>6.4112</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>dokumen_uji.pdf: AES-256-GCM</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1437152</v>
+      </c>
+      <c r="C12" t="n">
+        <v>7.9999</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>dokumen_uji.pdf: ChaCha20-Poly1305</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1437152</v>
+      </c>
+      <c r="C13" t="n">
+        <v>7.9999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>